<commit_message>
screener: relatório de 2026-08-08
</commit_message>
<xml_diff>
--- a/reports/screener_2026-08-08.xlsx
+++ b/reports/screener_2026-08-08.xlsx
@@ -1633,7 +1633,7 @@
         <v>-4.846816893197337</v>
       </c>
       <c r="BS5" t="n">
-        <v>-23.76550987166468</v>
+        <v>-23.76550462277683</v>
       </c>
       <c r="BT5" t="b">
         <v>1</v>
@@ -2326,7 +2326,7 @@
         <v>-15.98513225317606</v>
       </c>
       <c r="BS8" t="n">
-        <v>-43.15146077270641</v>
+        <v>-43.15145724236707</v>
       </c>
       <c r="BT8" t="b">
         <v>1</v>
@@ -3058,10 +3058,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>70.83</v>
+        <v>70.78</v>
       </c>
       <c r="F12" t="n">
-        <v>68.63</v>
+        <v>68.56</v>
       </c>
       <c r="G12" t="n">
         <v>83.33333333333333</v>
@@ -3077,7 +3077,7 @@
         <v>83.87</v>
       </c>
       <c r="L12" t="n">
-        <v>82.55</v>
+        <v>81.88</v>
       </c>
       <c r="M12" t="n">
         <v>11</v>
@@ -4837,12 +4837,12 @@
       </c>
       <c r="BL19" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="BM19" t="inlineStr">
         <is>
-          <t>última</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="BN19" t="inlineStr"/>
@@ -5681,7 +5681,7 @@
         <v>1</v>
       </c>
       <c r="AM23" t="n">
-        <v>18018230272</v>
+        <v>18537529344</v>
       </c>
       <c r="AN23" t="n">
         <v>6.56</v>
@@ -7883,10 +7883,10 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>63.17</v>
+        <v>63.1</v>
       </c>
       <c r="F33" t="n">
-        <v>63.73</v>
+        <v>63.64</v>
       </c>
       <c r="G33" t="n">
         <v>60</v>
@@ -7900,7 +7900,7 @@
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
-        <v>83.22</v>
+        <v>82.55</v>
       </c>
       <c r="M33" t="n">
         <v>32</v>
@@ -8748,7 +8748,7 @@
         <v>-2.664893844804339</v>
       </c>
       <c r="BS36" t="n">
-        <v>-19.62749400029969</v>
+        <v>-19.62750247023346</v>
       </c>
       <c r="BT36" t="b">
         <v>1</v>
@@ -10014,7 +10014,7 @@
         <v>1</v>
       </c>
       <c r="AM42" t="n">
-        <v>171916886016</v>
+        <v>165008867328</v>
       </c>
       <c r="AN42" t="n">
         <v>6.48</v>
@@ -10108,7 +10108,7 @@
         <v>-8.195107168235239</v>
       </c>
       <c r="BS42" t="n">
-        <v>-16.7134172222279</v>
+        <v>-16.71342624530195</v>
       </c>
       <c r="BT42" t="b">
         <v>1</v>
@@ -10147,10 +10147,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>59.87</v>
+        <v>59.91</v>
       </c>
       <c r="F43" t="n">
-        <v>55.73</v>
+        <v>55.78</v>
       </c>
       <c r="G43" t="n">
         <v>83.33333333333333</v>
@@ -10160,7 +10160,7 @@
         <v>78.54000000000001</v>
       </c>
       <c r="J43" t="n">
-        <v>18.14</v>
+        <v>18.34</v>
       </c>
       <c r="K43" t="n">
         <v>54.08</v>
@@ -12629,7 +12629,7 @@
         <v>-0.2309433623165158</v>
       </c>
       <c r="BS53" t="n">
-        <v>-19.41669381125899</v>
+        <v>-19.41668752521939</v>
       </c>
       <c r="BT53" t="b">
         <v>1</v>
@@ -12649,45 +12649,45 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BMOB3</t>
+          <t>WEGE3</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SMALL11</t>
+          <t>BOVA11</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SMALL11</t>
+          <t>BOVA11</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>57.26</v>
+        <v>57.31</v>
       </c>
       <c r="F54" t="n">
-        <v>52.65</v>
+        <v>55.66</v>
       </c>
       <c r="G54" t="n">
-        <v>83.33333333333333</v>
+        <v>66.66666666666667</v>
       </c>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="n">
-        <v>56.34</v>
+        <v>86.20999999999999</v>
       </c>
       <c r="J54" t="n">
-        <v>27.79</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="K54" t="n">
-        <v>74.59</v>
+        <v>63.66</v>
       </c>
       <c r="L54" t="n">
-        <v>54.36</v>
+        <v>20.13</v>
       </c>
       <c r="M54" t="n">
         <v>53</v>
@@ -12698,7 +12698,7 @@
         </is>
       </c>
       <c r="O54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P54" t="n">
         <v>7</v>
@@ -12721,13 +12721,13 @@
         <v>1</v>
       </c>
       <c r="X54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y54" t="b">
         <v>1</v>
       </c>
       <c r="Z54" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA54" t="n">
         <v>6</v>
@@ -12742,17 +12742,17 @@
         <v>1</v>
       </c>
       <c r="AE54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG54" t="inlineStr"/>
       <c r="AH54" t="b">
         <v>1</v>
       </c>
       <c r="AI54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ54" t="b">
         <v>1</v>
@@ -12762,83 +12762,83 @@
         <v>1</v>
       </c>
       <c r="AM54" t="n">
-        <v>1902465664</v>
+        <v>201903325184</v>
       </c>
       <c r="AN54" t="n">
-        <v>12.25</v>
+        <v>32.3</v>
       </c>
       <c r="AO54" t="n">
-        <v>2.01</v>
+        <v>10.71</v>
       </c>
       <c r="AP54" t="n">
-        <v>9.34</v>
+        <v>4.17</v>
       </c>
       <c r="AQ54" t="n">
-        <v>5.97</v>
+        <v>2.33</v>
       </c>
       <c r="AR54" t="n">
-        <v>16.39</v>
+        <v>33.16</v>
       </c>
       <c r="AS54" t="n">
-        <v>10.11</v>
+        <v>24.33</v>
       </c>
       <c r="AT54" t="n">
-        <v>8.91</v>
+        <v>15.58</v>
       </c>
       <c r="AU54" t="inlineStr"/>
       <c r="AV54" t="n">
-        <v>1.78</v>
+        <v>1.59</v>
       </c>
       <c r="AW54" t="n">
-        <v>0.05</v>
+        <v>0.29</v>
       </c>
       <c r="AX54" t="n">
-        <v>2.79</v>
+        <v>3.94</v>
       </c>
       <c r="AY54" t="n">
-        <v>22.85000038146973</v>
+        <v>48.11999893188477</v>
       </c>
       <c r="AZ54" t="n">
-        <v>9.75</v>
+        <v>8.01</v>
       </c>
       <c r="BA54" t="n">
-        <v>14.84</v>
+        <v>14.86</v>
       </c>
       <c r="BB54" t="n">
-        <v>20.28</v>
+        <v>19.74</v>
       </c>
       <c r="BC54" t="n">
-        <v>21.84</v>
+        <v>12.27</v>
       </c>
       <c r="BD54" t="n">
-        <v>19.34</v>
+        <v>15.69</v>
       </c>
       <c r="BE54" t="n">
-        <v>17.21</v>
+        <v>14.11</v>
       </c>
       <c r="BF54" t="n">
-        <v>19.34</v>
+        <v>14.86</v>
       </c>
       <c r="BG54" t="n">
-        <v>17.41</v>
+        <v>13.37</v>
       </c>
       <c r="BH54" t="n">
         <v>5</v>
       </c>
       <c r="BI54" t="n">
-        <v>-23.81</v>
+        <v>-72.20999999999999</v>
       </c>
       <c r="BJ54" t="n">
-        <v>-24.68</v>
+        <v>-70.67</v>
       </c>
       <c r="BK54" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="BL54" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="BM54" t="inlineStr">
@@ -12854,13 +12854,13 @@
         </is>
       </c>
       <c r="BQ54" t="n">
-        <v>24.03000068664551</v>
+        <v>49.16999816894531</v>
       </c>
       <c r="BR54" t="n">
-        <v>-4.910529635696426</v>
+        <v>-2.135446972059685</v>
       </c>
       <c r="BS54" t="n">
-        <v>-19.57500722208761</v>
+        <v>-11.35736832508161</v>
       </c>
       <c r="BT54" t="b">
         <v>1</v>
@@ -12873,52 +12873,52 @@
       </c>
       <c r="BW54" t="inlineStr">
         <is>
-          <t>sem sinal (Lateral; sem novo topo (-4.9%))</t>
+          <t>sem sinal (Lateral; sem novo topo (-2.1%))</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>WEGE3</t>
+          <t>BMOB3</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>BOVA11</t>
+          <t>SMALL11</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>BOVA11</t>
+          <t>SMALL11</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="E55" t="n">
         <v>57.26</v>
       </c>
       <c r="F55" t="n">
-        <v>55.6</v>
+        <v>52.65</v>
       </c>
       <c r="G55" t="n">
-        <v>66.66666666666667</v>
+        <v>83.33333333333333</v>
       </c>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="n">
-        <v>86.20999999999999</v>
+        <v>56.34</v>
       </c>
       <c r="J55" t="n">
-        <v>8.25</v>
+        <v>27.79</v>
       </c>
       <c r="K55" t="n">
-        <v>63.66</v>
+        <v>74.59</v>
       </c>
       <c r="L55" t="n">
-        <v>20.13</v>
+        <v>54.36</v>
       </c>
       <c r="M55" t="n">
         <v>54</v>
@@ -12929,7 +12929,7 @@
         </is>
       </c>
       <c r="O55" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P55" t="n">
         <v>7</v>
@@ -12952,13 +12952,13 @@
         <v>1</v>
       </c>
       <c r="X55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y55" t="b">
         <v>1</v>
       </c>
       <c r="Z55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AA55" t="n">
         <v>6</v>
@@ -12973,17 +12973,17 @@
         <v>1</v>
       </c>
       <c r="AE55" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG55" t="inlineStr"/>
       <c r="AH55" t="b">
         <v>1</v>
       </c>
       <c r="AI55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ55" t="b">
         <v>1</v>
@@ -12993,83 +12993,83 @@
         <v>1</v>
       </c>
       <c r="AM55" t="n">
-        <v>201903325184</v>
+        <v>1902465664</v>
       </c>
       <c r="AN55" t="n">
-        <v>32.3</v>
+        <v>12.25</v>
       </c>
       <c r="AO55" t="n">
-        <v>10.71</v>
+        <v>2.01</v>
       </c>
       <c r="AP55" t="n">
-        <v>4.17</v>
+        <v>9.34</v>
       </c>
       <c r="AQ55" t="n">
-        <v>2.33</v>
+        <v>5.97</v>
       </c>
       <c r="AR55" t="n">
-        <v>33.16</v>
+        <v>16.39</v>
       </c>
       <c r="AS55" t="n">
-        <v>24.33</v>
+        <v>10.11</v>
       </c>
       <c r="AT55" t="n">
-        <v>15.58</v>
+        <v>8.91</v>
       </c>
       <c r="AU55" t="inlineStr"/>
       <c r="AV55" t="n">
-        <v>1.59</v>
+        <v>1.78</v>
       </c>
       <c r="AW55" t="n">
-        <v>0.29</v>
+        <v>0.05</v>
       </c>
       <c r="AX55" t="n">
-        <v>3.94</v>
+        <v>2.79</v>
       </c>
       <c r="AY55" t="n">
-        <v>48.11999893188477</v>
+        <v>22.85000038146973</v>
       </c>
       <c r="AZ55" t="n">
-        <v>8.01</v>
+        <v>9.75</v>
       </c>
       <c r="BA55" t="n">
-        <v>14.86</v>
+        <v>14.84</v>
       </c>
       <c r="BB55" t="n">
-        <v>19.74</v>
+        <v>20.28</v>
       </c>
       <c r="BC55" t="n">
-        <v>12.27</v>
+        <v>21.84</v>
       </c>
       <c r="BD55" t="n">
-        <v>15.69</v>
+        <v>19.34</v>
       </c>
       <c r="BE55" t="n">
-        <v>14.11</v>
+        <v>17.21</v>
       </c>
       <c r="BF55" t="n">
-        <v>14.86</v>
+        <v>19.34</v>
       </c>
       <c r="BG55" t="n">
-        <v>13.37</v>
+        <v>17.41</v>
       </c>
       <c r="BH55" t="n">
         <v>5</v>
       </c>
       <c r="BI55" t="n">
-        <v>-72.20999999999999</v>
+        <v>-23.81</v>
       </c>
       <c r="BJ55" t="n">
-        <v>-70.67</v>
+        <v>-24.68</v>
       </c>
       <c r="BK55" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="BL55" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="BM55" t="inlineStr">
@@ -13085,13 +13085,13 @@
         </is>
       </c>
       <c r="BQ55" t="n">
-        <v>49.16999816894531</v>
+        <v>24.03000068664551</v>
       </c>
       <c r="BR55" t="n">
-        <v>-2.135446972059685</v>
+        <v>-4.910529635696426</v>
       </c>
       <c r="BS55" t="n">
-        <v>-11.35736832508161</v>
+        <v>-19.57500722208761</v>
       </c>
       <c r="BT55" t="b">
         <v>1</v>
@@ -13104,7 +13104,7 @@
       </c>
       <c r="BW55" t="inlineStr">
         <is>
-          <t>sem sinal (Lateral; sem novo topo (-2.1%))</t>
+          <t>sem sinal (Lateral; sem novo topo (-4.9%))</t>
         </is>
       </c>
     </row>
@@ -13143,13 +13143,13 @@
         <v>75.51000000000001</v>
       </c>
       <c r="J56" t="n">
-        <v>32.89</v>
+        <v>32.07</v>
       </c>
       <c r="K56" t="n">
         <v>22.81</v>
       </c>
       <c r="L56" t="n">
-        <v>81.88</v>
+        <v>83.89</v>
       </c>
       <c r="M56" t="n">
         <v>55</v>
@@ -13236,7 +13236,7 @@
         <v>8.33</v>
       </c>
       <c r="AQ56" t="n">
-        <v>10.06</v>
+        <v>10.3</v>
       </c>
       <c r="AR56" t="n">
         <v>23.72</v>
@@ -13255,43 +13255,43 @@
         <v>1.43</v>
       </c>
       <c r="AX56" t="n">
-        <v>3.85</v>
+        <v>4.89</v>
       </c>
       <c r="AY56" t="n">
         <v>44.79999923706055</v>
       </c>
       <c r="AZ56" t="n">
-        <v>32.21</v>
+        <v>32.96</v>
       </c>
       <c r="BA56" t="n">
-        <v>39.54</v>
+        <v>38.61</v>
       </c>
       <c r="BB56" t="n">
-        <v>43.84</v>
+        <v>41.84</v>
       </c>
       <c r="BC56" t="n">
         <v>48.76</v>
       </c>
       <c r="BD56" t="n">
-        <v>61.97</v>
+        <v>60.65</v>
       </c>
       <c r="BE56" t="n">
-        <v>45.26</v>
+        <v>44.56</v>
       </c>
       <c r="BF56" t="n">
-        <v>43.84</v>
+        <v>41.84</v>
       </c>
       <c r="BG56" t="n">
-        <v>39.46</v>
+        <v>37.66</v>
       </c>
       <c r="BH56" t="n">
         <v>5</v>
       </c>
       <c r="BI56" t="n">
-        <v>-11.93</v>
+        <v>-15.94</v>
       </c>
       <c r="BJ56" t="n">
-        <v>1.03</v>
+        <v>-0.53</v>
       </c>
       <c r="BK56" t="inlineStr">
         <is>
@@ -14232,7 +14232,7 @@
         <v>-5.60574072640605</v>
       </c>
       <c r="BS60" t="n">
-        <v>-16.35821943150735</v>
+        <v>-16.35820625379285</v>
       </c>
       <c r="BT60" t="b">
         <v>1</v>
@@ -15387,7 +15387,7 @@
         <v>-14.94578145537126</v>
       </c>
       <c r="BS65" t="n">
-        <v>-25.82515452490343</v>
+        <v>-25.82514761546183</v>
       </c>
       <c r="BT65" t="b">
         <v>1</v>
@@ -18476,7 +18476,7 @@
         <v>-4.846816893197337</v>
       </c>
       <c r="BS5" t="n">
-        <v>-23.76550987166468</v>
+        <v>-23.76550462277683</v>
       </c>
       <c r="BT5" t="b">
         <v>1</v>
@@ -19169,7 +19169,7 @@
         <v>-15.98513225317606</v>
       </c>
       <c r="BS8" t="n">
-        <v>-43.15146077270641</v>
+        <v>-43.15145724236707</v>
       </c>
       <c r="BT8" t="b">
         <v>1</v>
@@ -19901,10 +19901,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>70.83</v>
+        <v>70.78</v>
       </c>
       <c r="F12" t="n">
-        <v>68.63</v>
+        <v>68.56</v>
       </c>
       <c r="G12" t="n">
         <v>83.33333333333333</v>
@@ -19920,7 +19920,7 @@
         <v>83.87</v>
       </c>
       <c r="L12" t="n">
-        <v>82.55</v>
+        <v>81.88</v>
       </c>
       <c r="M12" t="n">
         <v>11</v>
@@ -21680,12 +21680,12 @@
       </c>
       <c r="BL19" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="BM19" t="inlineStr">
         <is>
-          <t>última</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="BN19" t="inlineStr"/>
@@ -22524,7 +22524,7 @@
         <v>1</v>
       </c>
       <c r="AM23" t="n">
-        <v>18018230272</v>
+        <v>18537529344</v>
       </c>
       <c r="AN23" t="n">
         <v>6.56</v>
@@ -24726,10 +24726,10 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>63.17</v>
+        <v>63.1</v>
       </c>
       <c r="F33" t="n">
-        <v>63.73</v>
+        <v>63.64</v>
       </c>
       <c r="G33" t="n">
         <v>60</v>
@@ -24743,7 +24743,7 @@
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
-        <v>83.22</v>
+        <v>82.55</v>
       </c>
       <c r="M33" t="n">
         <v>32</v>
@@ -25591,7 +25591,7 @@
         <v>-2.664893844804339</v>
       </c>
       <c r="BS36" t="n">
-        <v>-19.62749400029969</v>
+        <v>-19.62750247023346</v>
       </c>
       <c r="BT36" t="b">
         <v>1</v>
@@ -26857,7 +26857,7 @@
         <v>1</v>
       </c>
       <c r="AM42" t="n">
-        <v>171916886016</v>
+        <v>165008867328</v>
       </c>
       <c r="AN42" t="n">
         <v>6.48</v>
@@ -26951,7 +26951,7 @@
         <v>-8.195107168235239</v>
       </c>
       <c r="BS42" t="n">
-        <v>-16.7134172222279</v>
+        <v>-16.71342624530195</v>
       </c>
       <c r="BT42" t="b">
         <v>1</v>
@@ -26990,10 +26990,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>59.87</v>
+        <v>59.91</v>
       </c>
       <c r="F43" t="n">
-        <v>55.73</v>
+        <v>55.78</v>
       </c>
       <c r="G43" t="n">
         <v>83.33333333333333</v>
@@ -27003,7 +27003,7 @@
         <v>78.54000000000001</v>
       </c>
       <c r="J43" t="n">
-        <v>18.14</v>
+        <v>18.34</v>
       </c>
       <c r="K43" t="n">
         <v>54.08</v>
@@ -29472,7 +29472,7 @@
         <v>-0.2309433623165158</v>
       </c>
       <c r="BS53" t="n">
-        <v>-19.41669381125899</v>
+        <v>-19.41668752521939</v>
       </c>
       <c r="BT53" t="b">
         <v>1</v>
@@ -29492,45 +29492,45 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BMOB3</t>
+          <t>WEGE3</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SMALL11</t>
+          <t>BOVA11</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SMALL11</t>
+          <t>BOVA11</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>57.26</v>
+        <v>57.31</v>
       </c>
       <c r="F54" t="n">
-        <v>52.65</v>
+        <v>55.66</v>
       </c>
       <c r="G54" t="n">
-        <v>83.33333333333333</v>
+        <v>66.66666666666667</v>
       </c>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="n">
-        <v>56.34</v>
+        <v>86.20999999999999</v>
       </c>
       <c r="J54" t="n">
-        <v>27.79</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="K54" t="n">
-        <v>74.59</v>
+        <v>63.66</v>
       </c>
       <c r="L54" t="n">
-        <v>54.36</v>
+        <v>20.13</v>
       </c>
       <c r="M54" t="n">
         <v>53</v>
@@ -29541,7 +29541,7 @@
         </is>
       </c>
       <c r="O54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P54" t="n">
         <v>7</v>
@@ -29564,13 +29564,13 @@
         <v>1</v>
       </c>
       <c r="X54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y54" t="b">
         <v>1</v>
       </c>
       <c r="Z54" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA54" t="n">
         <v>6</v>
@@ -29585,17 +29585,17 @@
         <v>1</v>
       </c>
       <c r="AE54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG54" t="inlineStr"/>
       <c r="AH54" t="b">
         <v>1</v>
       </c>
       <c r="AI54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ54" t="b">
         <v>1</v>
@@ -29605,83 +29605,83 @@
         <v>1</v>
       </c>
       <c r="AM54" t="n">
-        <v>1902465664</v>
+        <v>201903325184</v>
       </c>
       <c r="AN54" t="n">
-        <v>12.25</v>
+        <v>32.3</v>
       </c>
       <c r="AO54" t="n">
-        <v>2.01</v>
+        <v>10.71</v>
       </c>
       <c r="AP54" t="n">
-        <v>9.34</v>
+        <v>4.17</v>
       </c>
       <c r="AQ54" t="n">
-        <v>5.97</v>
+        <v>2.33</v>
       </c>
       <c r="AR54" t="n">
-        <v>16.39</v>
+        <v>33.16</v>
       </c>
       <c r="AS54" t="n">
-        <v>10.11</v>
+        <v>24.33</v>
       </c>
       <c r="AT54" t="n">
-        <v>8.91</v>
+        <v>15.58</v>
       </c>
       <c r="AU54" t="inlineStr"/>
       <c r="AV54" t="n">
-        <v>1.78</v>
+        <v>1.59</v>
       </c>
       <c r="AW54" t="n">
-        <v>0.05</v>
+        <v>0.29</v>
       </c>
       <c r="AX54" t="n">
-        <v>2.79</v>
+        <v>3.94</v>
       </c>
       <c r="AY54" t="n">
-        <v>22.85000038146973</v>
+        <v>48.11999893188477</v>
       </c>
       <c r="AZ54" t="n">
-        <v>9.75</v>
+        <v>8.01</v>
       </c>
       <c r="BA54" t="n">
-        <v>14.84</v>
+        <v>14.86</v>
       </c>
       <c r="BB54" t="n">
-        <v>20.28</v>
+        <v>19.74</v>
       </c>
       <c r="BC54" t="n">
-        <v>21.84</v>
+        <v>12.27</v>
       </c>
       <c r="BD54" t="n">
-        <v>19.34</v>
+        <v>15.69</v>
       </c>
       <c r="BE54" t="n">
-        <v>17.21</v>
+        <v>14.11</v>
       </c>
       <c r="BF54" t="n">
-        <v>19.34</v>
+        <v>14.86</v>
       </c>
       <c r="BG54" t="n">
-        <v>17.41</v>
+        <v>13.37</v>
       </c>
       <c r="BH54" t="n">
         <v>5</v>
       </c>
       <c r="BI54" t="n">
-        <v>-23.81</v>
+        <v>-72.20999999999999</v>
       </c>
       <c r="BJ54" t="n">
-        <v>-24.68</v>
+        <v>-70.67</v>
       </c>
       <c r="BK54" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="BL54" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="BM54" t="inlineStr">
@@ -29697,13 +29697,13 @@
         </is>
       </c>
       <c r="BQ54" t="n">
-        <v>24.03000068664551</v>
+        <v>49.16999816894531</v>
       </c>
       <c r="BR54" t="n">
-        <v>-4.910529635696426</v>
+        <v>-2.135446972059685</v>
       </c>
       <c r="BS54" t="n">
-        <v>-19.57500722208761</v>
+        <v>-11.35736832508161</v>
       </c>
       <c r="BT54" t="b">
         <v>1</v>
@@ -29716,52 +29716,52 @@
       </c>
       <c r="BW54" t="inlineStr">
         <is>
-          <t>sem sinal (Lateral; sem novo topo (-4.9%))</t>
+          <t>sem sinal (Lateral; sem novo topo (-2.1%))</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>WEGE3</t>
+          <t>BMOB3</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>BOVA11</t>
+          <t>SMALL11</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>BOVA11</t>
+          <t>SMALL11</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="E55" t="n">
         <v>57.26</v>
       </c>
       <c r="F55" t="n">
-        <v>55.6</v>
+        <v>52.65</v>
       </c>
       <c r="G55" t="n">
-        <v>66.66666666666667</v>
+        <v>83.33333333333333</v>
       </c>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="n">
-        <v>86.20999999999999</v>
+        <v>56.34</v>
       </c>
       <c r="J55" t="n">
-        <v>8.25</v>
+        <v>27.79</v>
       </c>
       <c r="K55" t="n">
-        <v>63.66</v>
+        <v>74.59</v>
       </c>
       <c r="L55" t="n">
-        <v>20.13</v>
+        <v>54.36</v>
       </c>
       <c r="M55" t="n">
         <v>54</v>
@@ -29772,7 +29772,7 @@
         </is>
       </c>
       <c r="O55" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P55" t="n">
         <v>7</v>
@@ -29795,13 +29795,13 @@
         <v>1</v>
       </c>
       <c r="X55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y55" t="b">
         <v>1</v>
       </c>
       <c r="Z55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AA55" t="n">
         <v>6</v>
@@ -29816,17 +29816,17 @@
         <v>1</v>
       </c>
       <c r="AE55" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG55" t="inlineStr"/>
       <c r="AH55" t="b">
         <v>1</v>
       </c>
       <c r="AI55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ55" t="b">
         <v>1</v>
@@ -29836,83 +29836,83 @@
         <v>1</v>
       </c>
       <c r="AM55" t="n">
-        <v>201903325184</v>
+        <v>1902465664</v>
       </c>
       <c r="AN55" t="n">
-        <v>32.3</v>
+        <v>12.25</v>
       </c>
       <c r="AO55" t="n">
-        <v>10.71</v>
+        <v>2.01</v>
       </c>
       <c r="AP55" t="n">
-        <v>4.17</v>
+        <v>9.34</v>
       </c>
       <c r="AQ55" t="n">
-        <v>2.33</v>
+        <v>5.97</v>
       </c>
       <c r="AR55" t="n">
-        <v>33.16</v>
+        <v>16.39</v>
       </c>
       <c r="AS55" t="n">
-        <v>24.33</v>
+        <v>10.11</v>
       </c>
       <c r="AT55" t="n">
-        <v>15.58</v>
+        <v>8.91</v>
       </c>
       <c r="AU55" t="inlineStr"/>
       <c r="AV55" t="n">
-        <v>1.59</v>
+        <v>1.78</v>
       </c>
       <c r="AW55" t="n">
-        <v>0.29</v>
+        <v>0.05</v>
       </c>
       <c r="AX55" t="n">
-        <v>3.94</v>
+        <v>2.79</v>
       </c>
       <c r="AY55" t="n">
-        <v>48.11999893188477</v>
+        <v>22.85000038146973</v>
       </c>
       <c r="AZ55" t="n">
-        <v>8.01</v>
+        <v>9.75</v>
       </c>
       <c r="BA55" t="n">
-        <v>14.86</v>
+        <v>14.84</v>
       </c>
       <c r="BB55" t="n">
-        <v>19.74</v>
+        <v>20.28</v>
       </c>
       <c r="BC55" t="n">
-        <v>12.27</v>
+        <v>21.84</v>
       </c>
       <c r="BD55" t="n">
-        <v>15.69</v>
+        <v>19.34</v>
       </c>
       <c r="BE55" t="n">
-        <v>14.11</v>
+        <v>17.21</v>
       </c>
       <c r="BF55" t="n">
-        <v>14.86</v>
+        <v>19.34</v>
       </c>
       <c r="BG55" t="n">
-        <v>13.37</v>
+        <v>17.41</v>
       </c>
       <c r="BH55" t="n">
         <v>5</v>
       </c>
       <c r="BI55" t="n">
-        <v>-72.20999999999999</v>
+        <v>-23.81</v>
       </c>
       <c r="BJ55" t="n">
-        <v>-70.67</v>
+        <v>-24.68</v>
       </c>
       <c r="BK55" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="BL55" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="BM55" t="inlineStr">
@@ -29928,13 +29928,13 @@
         </is>
       </c>
       <c r="BQ55" t="n">
-        <v>49.16999816894531</v>
+        <v>24.03000068664551</v>
       </c>
       <c r="BR55" t="n">
-        <v>-2.135446972059685</v>
+        <v>-4.910529635696426</v>
       </c>
       <c r="BS55" t="n">
-        <v>-11.35736832508161</v>
+        <v>-19.57500722208761</v>
       </c>
       <c r="BT55" t="b">
         <v>1</v>
@@ -29947,7 +29947,7 @@
       </c>
       <c r="BW55" t="inlineStr">
         <is>
-          <t>sem sinal (Lateral; sem novo topo (-2.1%))</t>
+          <t>sem sinal (Lateral; sem novo topo (-4.9%))</t>
         </is>
       </c>
     </row>
@@ -29986,13 +29986,13 @@
         <v>75.51000000000001</v>
       </c>
       <c r="J56" t="n">
-        <v>32.89</v>
+        <v>32.07</v>
       </c>
       <c r="K56" t="n">
         <v>22.81</v>
       </c>
       <c r="L56" t="n">
-        <v>81.88</v>
+        <v>83.89</v>
       </c>
       <c r="M56" t="n">
         <v>55</v>
@@ -30079,7 +30079,7 @@
         <v>8.33</v>
       </c>
       <c r="AQ56" t="n">
-        <v>10.06</v>
+        <v>10.3</v>
       </c>
       <c r="AR56" t="n">
         <v>23.72</v>
@@ -30098,43 +30098,43 @@
         <v>1.43</v>
       </c>
       <c r="AX56" t="n">
-        <v>3.85</v>
+        <v>4.89</v>
       </c>
       <c r="AY56" t="n">
         <v>44.79999923706055</v>
       </c>
       <c r="AZ56" t="n">
-        <v>32.21</v>
+        <v>32.96</v>
       </c>
       <c r="BA56" t="n">
-        <v>39.54</v>
+        <v>38.61</v>
       </c>
       <c r="BB56" t="n">
-        <v>43.84</v>
+        <v>41.84</v>
       </c>
       <c r="BC56" t="n">
         <v>48.76</v>
       </c>
       <c r="BD56" t="n">
-        <v>61.97</v>
+        <v>60.65</v>
       </c>
       <c r="BE56" t="n">
-        <v>45.26</v>
+        <v>44.56</v>
       </c>
       <c r="BF56" t="n">
-        <v>43.84</v>
+        <v>41.84</v>
       </c>
       <c r="BG56" t="n">
-        <v>39.46</v>
+        <v>37.66</v>
       </c>
       <c r="BH56" t="n">
         <v>5</v>
       </c>
       <c r="BI56" t="n">
-        <v>-11.93</v>
+        <v>-15.94</v>
       </c>
       <c r="BJ56" t="n">
-        <v>1.03</v>
+        <v>-0.53</v>
       </c>
       <c r="BK56" t="inlineStr">
         <is>
@@ -31075,7 +31075,7 @@
         <v>-5.60574072640605</v>
       </c>
       <c r="BS60" t="n">
-        <v>-16.35821943150735</v>
+        <v>-16.35820625379285</v>
       </c>
       <c r="BT60" t="b">
         <v>1</v>
@@ -32230,7 +32230,7 @@
         <v>-14.94578145537126</v>
       </c>
       <c r="BS65" t="n">
-        <v>-25.82515452490343</v>
+        <v>-25.82514761546183</v>
       </c>
       <c r="BT65" t="b">
         <v>1</v>
@@ -35019,10 +35019,10 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>50.28</v>
+        <v>50.32</v>
       </c>
       <c r="F78" t="n">
-        <v>53.27</v>
+        <v>53.32</v>
       </c>
       <c r="G78" t="n">
         <v>33.33333333333334</v>
@@ -35032,7 +35032,7 @@
         <v>45.05</v>
       </c>
       <c r="J78" t="n">
-        <v>60.3</v>
+        <v>60.5</v>
       </c>
       <c r="K78" t="n">
         <v>46.98</v>
@@ -35246,10 +35246,10 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>50.11</v>
+        <v>50.05</v>
       </c>
       <c r="F79" t="n">
-        <v>50.13</v>
+        <v>50.06</v>
       </c>
       <c r="G79" t="n">
         <v>50</v>
@@ -35265,7 +35265,7 @@
         <v>42.11</v>
       </c>
       <c r="L79" t="n">
-        <v>83.89</v>
+        <v>83.22</v>
       </c>
       <c r="M79" t="n">
         <v>78</v>
@@ -36698,7 +36698,7 @@
         <v>1</v>
       </c>
       <c r="AM85" t="n">
-        <v>13472881664</v>
+        <v>13473802240</v>
       </c>
       <c r="AN85" t="n">
         <v>14.53</v>
@@ -36792,7 +36792,7 @@
         <v>-2.285089473123469</v>
       </c>
       <c r="BS85" t="n">
-        <v>-17.85090042584634</v>
+        <v>-17.850910086273</v>
       </c>
       <c r="BT85" t="b">
         <v>0</v>
@@ -37913,7 +37913,7 @@
         <v>-1.900235700265374</v>
       </c>
       <c r="BS90" t="n">
-        <v>-15.22971914757722</v>
+        <v>-15.22972761158513</v>
       </c>
       <c r="BT90" t="b">
         <v>0</v>
@@ -40617,7 +40617,7 @@
         <v>-2.411569511092404</v>
       </c>
       <c r="BS102" t="n">
-        <v>-25.49989727527226</v>
+        <v>-25.49988843235376</v>
       </c>
       <c r="BT102" t="b">
         <v>0</v>
@@ -44579,7 +44579,7 @@
         <v>-9.242822111007619</v>
       </c>
       <c r="BS120" t="n">
-        <v>-19.44250955845246</v>
+        <v>-19.44251454422593</v>
       </c>
       <c r="BT120" t="b">
         <v>0</v>
@@ -45656,7 +45656,7 @@
         <v>-7.69230636971937</v>
       </c>
       <c r="BS125" t="n">
-        <v>-54.87060603413229</v>
+        <v>-54.87060095233498</v>
       </c>
       <c r="BT125" t="b">
         <v>0</v>
@@ -46370,10 +46370,10 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>34.58</v>
+        <v>34.62</v>
       </c>
       <c r="F129" t="n">
-        <v>34.8</v>
+        <v>34.85</v>
       </c>
       <c r="G129" t="n">
         <v>33.33333333333334</v>
@@ -46383,7 +46383,7 @@
         <v>49.38</v>
       </c>
       <c r="J129" t="n">
-        <v>27.3</v>
+        <v>27.51</v>
       </c>
       <c r="K129" t="n">
         <v>22.05</v>

</xml_diff>